<commit_message>
Update with new thermal model option
</commit_message>
<xml_diff>
--- a/Selected Switch Model/GaN Data Check.xlsx
+++ b/Selected Switch Model/GaN Data Check.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Selected Switch Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A99C2DE-9ED6-4EA4-88F1-D2ECD1BF08CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C56890-BF3E-4620-9FE2-536C6E191B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -830,6 +830,10 @@
         <f t="shared" si="3"/>
         <v>0.51724137931034475</v>
       </c>
+      <c r="Y3" s="2">
+        <f>9.7*(0.5+0.6)</f>
+        <v>10.67</v>
+      </c>
       <c r="Z3" s="2">
         <v>2.5000000000000001E-2</v>
       </c>

</xml_diff>